<commit_message>
Date: 15 Apr 2026
</commit_message>
<xml_diff>
--- a/MyAtuomationProject/ExcelFiles/LoginData.xlsx
+++ b/MyAtuomationProject/ExcelFiles/LoginData.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="18">
   <si>
     <t>User Name</t>
   </si>
@@ -31,9 +31,6 @@
     <t>secret_sauce</t>
   </si>
   <si>
-    <t>Not Run</t>
-  </si>
-  <si>
     <t>Dhanashri</t>
   </si>
   <si>
@@ -61,7 +58,16 @@
     <t>Product</t>
   </si>
   <si>
-    <t>NULL</t>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Sauce Labs Backpack</t>
+  </si>
+  <si>
+    <t>Epic sadface: Username and password do not match any user in this service</t>
   </si>
 </sst>
 </file>
@@ -410,7 +416,8 @@
     <col min="1" max="1" width="23.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="1"/>
+    <col min="4" max="4" width="68.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -424,7 +431,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -435,80 +442,80 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>7</v>
-      </c>
       <c r="C3" s="1" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="C5" s="1" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="C7" s="1" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>